<commit_message>
adding smoke test script
</commit_message>
<xml_diff>
--- a/EComProject/Test-Data/OnlineBookstoreTD.xlsx
+++ b/EComProject/Test-Data/OnlineBookstoreTD.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4507"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010"/>
+    <workbookView xWindow="0" yWindow="2520" windowWidth="14655" windowHeight="6540"/>
   </bookViews>
   <sheets>
     <sheet name="Search_module" sheetId="1" r:id="rId1"/>
@@ -12,6 +12,7 @@
     <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="125725"/>
+  <oleSize ref="A1"/>
 </workbook>
 </file>
 
@@ -21,7 +22,7 @@
     <t>BookName</t>
   </si>
   <si>
-    <t>like a love song</t>
+    <t>Like a Love Song</t>
   </si>
 </sst>
 </file>

</xml_diff>